<commit_message>
Blueberry Funded : SCANNED se defend sur ce qu'il a, pas sur son taux
Reponse d'Adedayo (service client Blueberry, 30/09) : le coupon affilie reste
a 30 %, sans negociation possible, mais il vaut sur TOUS les types de compte
et n'a pas de date de fin — la ou PRIME50 et PRIMEBG sont reserves aux comptes
Prime et expirent.

La fiche dit donc ce que le code a de particulier plutot que de se comparer a
un pourcentage qu'elle perdrait :
  - accroche : « Works on every account type, and it has no end date. » ;
  - pastille : « No expiry » ;
  - couts : une ligne « Public campaigns » qui explique, sans vendre les codes
    du partenaire, pourquoi ils ne remplacent pas celui-ci.

Confirme aussi : ni lien par plan, ni coupon pre-applique chez ce partenaire.
Le lien de tracking suffit a rattacher la vente.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/firms/blueberry-funded.xlsx
+++ b/data/firms/blueberry-funded.xlsx
@@ -1511,6 +1511,11 @@
           <t>accroche</t>
         </is>
       </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Works on every account type, and it has no end date.</t>
+        </is>
+      </c>
       <c r="D10" s="15" t="inlineStr">
         <is>
           <t>Une phrase courte pour le bandeau de campagne du site : ce que l'offre donne, en plus du pourcentage. Vide : le bandeau n'affiche que la remise.</t>
@@ -1545,6 +1550,11 @@
       <c r="A13" s="15" t="inlineStr">
         <is>
           <t>bonus</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>No expiry</t>
         </is>
       </c>
       <c r="D13" s="15" t="inlineStr">
@@ -2330,10 +2340,24 @@
       <c r="E6" s="16" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="23" t="n"/>
-      <c r="B7" s="16" t="n"/>
-      <c r="C7" s="16" t="n"/>
-      <c r="D7" s="16" t="n"/>
+      <c r="A7" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Public campaigns</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Prime only, dated</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Blueberry runs its own codes from time to time. They are limited to Prime accounts and to a deadline; SCANNED has neither limit and applies to every account type (confirmed by Blueberry support, 30 September 2026).</t>
+        </is>
+      </c>
       <c r="E7" s="16" t="n"/>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
/compare : « No expiry » retire de Blueberry Funded
Sa pastille etait la seule de la premiere rangee : elle ajoutait une ligne au
cadre promo, donc 32 px a toute la rangee (415 px contre 383 px pour la
suivante), et poussait les boutons de ses trois voisines vers le bas. Les deux
rangees s'alignent de nouveau, et le code promo retrouve la place qu'il a
partout ailleurs.

L'argument reste sur la fiche, ou il a de la place : « Works on every account
type, and it has no end date. »

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/firms/blueberry-funded.xlsx
+++ b/data/firms/blueberry-funded.xlsx
@@ -1552,11 +1552,6 @@
           <t>bonus</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>No expiry</t>
-        </is>
-      </c>
       <c r="D13" s="15" t="inlineStr">
         <is>
           <t>Deux ou trois mots pour ce que l'offre donne en plus du pourcentage (« +1 free reset »). Affiche en pastille sur la fiche et sur la carte /compare. Suit la campagne : il disparait avec elle.</t>

</xml_diff>